<commit_message>
small rework of user msg in progress
</commit_message>
<xml_diff>
--- a/3-Dev/DevApp/Input/scriptOk.xlsx
+++ b/3-Dev/DevApp/Input/scriptOk.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/Lexerow/Dev/LexerowSol/3-Dev/DevApp/Input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/Lexerow/Dev/Lexerow/3-Dev/DevApp/Input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_AD4DB114E441178AC67DF4536695FF58683EDF1B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{593FD673-A99D-42D9-875E-9C1090575790}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="11_AD4DB114E441178AC67DF4536695FF58683EDF1B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB4110BE-134C-4775-A726-1CB9CC283A65}"/>
   <bookViews>
-    <workbookView xWindow="2895" yWindow="2565" windowWidth="22935" windowHeight="13725" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>string</t>
   </si>
@@ -40,6 +40,12 @@
   </si>
   <si>
     <t>double</t>
+  </si>
+  <si>
+    <t>hello</t>
+  </si>
+  <si>
+    <t>bonjour</t>
   </si>
 </sst>
 </file>
@@ -359,7 +365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -390,6 +396,34 @@
         <v>54</v>
       </c>
     </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>34</v>
+      </c>
+      <c r="C3">
+        <v>12</v>
+      </c>
+      <c r="D3">
+        <v>45.23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>7</v>
+      </c>
+      <c r="C4">
+        <v>9</v>
+      </c>
+      <c r="D4">
+        <v>23.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>